<commit_message>
Just updated contribution and added documents
</commit_message>
<xml_diff>
--- a/docs/Product Backlog - SOEN 341.xlsx
+++ b/docs/Product Backlog - SOEN 341.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gagne\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{23A24889-1192-4112-8A16-D5EBA4173EB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6F9F9410-BE07-424C-94F0-C2310F4B2BD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" firstSheet="2" activeTab="2" xr2:uid="{9FF516DD-DD1A-4540-862E-5B2452513E79}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" firstSheet="1" activeTab="2" xr2:uid="{9FF516DD-DD1A-4540-862E-5B2452513E79}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover Page" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="81">
   <si>
     <t>The Cool Team</t>
   </si>
@@ -333,6 +333,24 @@
   </si>
   <si>
     <t>Wrote some Acceptance Tests for some User Stories by testing the platform. With help, did the calorie tracker</t>
+  </si>
+  <si>
+    <t>Worked on the refactoring and seperating the code into Model, View, Controller architecture</t>
+  </si>
+  <si>
+    <t>Setup the static analysis tool and fixed found bugs.</t>
+  </si>
+  <si>
+    <t>Helped with the refactoring
+Helped with the restructuring
+Helped with final reprot</t>
+  </si>
+  <si>
+    <t>Worked on the final report and presentation slides</t>
+  </si>
+  <si>
+    <t>Created unit tests for sprint 3 and 4 features
+Helped with the final report</t>
   </si>
 </sst>
 </file>
@@ -815,6 +833,24 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -849,24 +885,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1220,18 +1238,18 @@
   </cols>
   <sheetData>
     <row r="5" spans="6:9" x14ac:dyDescent="0.35">
-      <c r="F5" s="66" t="s">
+      <c r="F5" s="57" t="s">
         <v>0</v>
       </c>
-      <c r="G5" s="66"/>
-      <c r="H5" s="66"/>
-      <c r="I5" s="66"/>
+      <c r="G5" s="57"/>
+      <c r="H5" s="57"/>
+      <c r="I5" s="57"/>
     </row>
     <row r="6" spans="6:9" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="F6" s="66"/>
-      <c r="G6" s="66"/>
-      <c r="H6" s="66"/>
-      <c r="I6" s="66"/>
+      <c r="F6" s="57"/>
+      <c r="G6" s="57"/>
+      <c r="H6" s="57"/>
+      <c r="I6" s="57"/>
     </row>
     <row r="7" spans="6:9" ht="23.5" x14ac:dyDescent="0.55000000000000004">
       <c r="F7" s="52"/>
@@ -1240,60 +1258,60 @@
       <c r="I7" s="52"/>
     </row>
     <row r="8" spans="6:9" ht="23.5" x14ac:dyDescent="0.55000000000000004">
-      <c r="F8" s="67" t="s">
+      <c r="F8" s="58" t="s">
         <v>1</v>
       </c>
-      <c r="G8" s="67"/>
-      <c r="H8" s="67"/>
-      <c r="I8" s="67"/>
+      <c r="G8" s="58"/>
+      <c r="H8" s="58"/>
+      <c r="I8" s="58"/>
     </row>
     <row r="9" spans="6:9" ht="23.5" x14ac:dyDescent="0.55000000000000004">
-      <c r="F9" s="65" t="s">
+      <c r="F9" s="56" t="s">
         <v>2</v>
       </c>
-      <c r="G9" s="65"/>
-      <c r="H9" s="65"/>
-      <c r="I9" s="65"/>
+      <c r="G9" s="56"/>
+      <c r="H9" s="56"/>
+      <c r="I9" s="56"/>
     </row>
     <row r="10" spans="6:9" ht="23.5" x14ac:dyDescent="0.55000000000000004">
-      <c r="F10" s="65" t="s">
+      <c r="F10" s="56" t="s">
         <v>3</v>
       </c>
-      <c r="G10" s="65"/>
-      <c r="H10" s="65"/>
-      <c r="I10" s="65"/>
+      <c r="G10" s="56"/>
+      <c r="H10" s="56"/>
+      <c r="I10" s="56"/>
     </row>
     <row r="11" spans="6:9" ht="23.5" x14ac:dyDescent="0.55000000000000004">
-      <c r="F11" s="65" t="s">
+      <c r="F11" s="56" t="s">
         <v>4</v>
       </c>
-      <c r="G11" s="65"/>
-      <c r="H11" s="65"/>
-      <c r="I11" s="65"/>
+      <c r="G11" s="56"/>
+      <c r="H11" s="56"/>
+      <c r="I11" s="56"/>
     </row>
     <row r="12" spans="6:9" ht="23.5" x14ac:dyDescent="0.55000000000000004">
-      <c r="F12" s="65" t="s">
+      <c r="F12" s="56" t="s">
         <v>5</v>
       </c>
-      <c r="G12" s="65"/>
-      <c r="H12" s="65"/>
-      <c r="I12" s="65"/>
+      <c r="G12" s="56"/>
+      <c r="H12" s="56"/>
+      <c r="I12" s="56"/>
     </row>
     <row r="13" spans="6:9" ht="23.5" x14ac:dyDescent="0.55000000000000004">
-      <c r="F13" s="65" t="s">
+      <c r="F13" s="56" t="s">
         <v>6</v>
       </c>
-      <c r="G13" s="65"/>
-      <c r="H13" s="65"/>
-      <c r="I13" s="65"/>
+      <c r="G13" s="56"/>
+      <c r="H13" s="56"/>
+      <c r="I13" s="56"/>
     </row>
     <row r="14" spans="6:9" ht="23.5" x14ac:dyDescent="0.55000000000000004">
-      <c r="F14" s="65" t="s">
+      <c r="F14" s="56" t="s">
         <v>7</v>
       </c>
-      <c r="G14" s="65"/>
-      <c r="H14" s="65"/>
-      <c r="I14" s="65"/>
+      <c r="G14" s="56"/>
+      <c r="H14" s="56"/>
+      <c r="I14" s="56"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -1496,7 +1514,7 @@
         <v>34</v>
       </c>
       <c r="D7" s="25">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E7" s="25" t="s">
         <v>18</v>
@@ -1642,14 +1660,14 @@
       </c>
     </row>
     <row r="13" spans="1:8" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A13" s="68" t="s">
+      <c r="A13" s="53" t="s">
         <v>50</v>
       </c>
-      <c r="B13" s="69"/>
-      <c r="C13" s="70"/>
+      <c r="B13" s="54"/>
+      <c r="C13" s="55"/>
       <c r="D13" s="5">
         <f>SUM(D2:D12)</f>
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E13" s="2"/>
       <c r="F13" s="2"/>
@@ -1770,7 +1788,7 @@
       </c>
     </row>
     <row r="3" spans="1:7" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="55" t="s">
+      <c r="A3" s="61" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="6" t="s">
@@ -1785,14 +1803,16 @@
       <c r="E3" s="14">
         <v>5</v>
       </c>
-      <c r="F3" s="14"/>
+      <c r="F3" s="14">
+        <v>15</v>
+      </c>
       <c r="G3" s="11">
         <f>SUM(C3:F3)</f>
-        <v>15</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="97.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="56"/>
+      <c r="A4" s="62"/>
       <c r="B4" s="7" t="s">
         <v>57</v>
       </c>
@@ -1805,11 +1825,13 @@
       <c r="E4" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="F4" s="15"/>
+      <c r="F4" s="4" t="s">
+        <v>76</v>
+      </c>
       <c r="G4" s="12"/>
     </row>
     <row r="5" spans="1:7" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="57" t="s">
+      <c r="A5" s="63" t="s">
         <v>3</v>
       </c>
       <c r="B5" s="6" t="s">
@@ -1824,14 +1846,16 @@
       <c r="E5" s="14">
         <v>15</v>
       </c>
-      <c r="F5" s="14"/>
+      <c r="F5" s="14">
+        <v>10</v>
+      </c>
       <c r="G5" s="11">
         <f>SUM(C5:F5)</f>
-        <v>25</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="101.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="58"/>
+      <c r="A6" s="64"/>
       <c r="B6" s="7" t="s">
         <v>57</v>
       </c>
@@ -1844,11 +1868,13 @@
       <c r="E6" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="F6" s="15"/>
+      <c r="F6" s="15" t="s">
+        <v>77</v>
+      </c>
       <c r="G6" s="12"/>
     </row>
     <row r="7" spans="1:7" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="59" t="s">
+      <c r="A7" s="65" t="s">
         <v>5</v>
       </c>
       <c r="B7" s="6" t="s">
@@ -1863,14 +1889,16 @@
       <c r="E7" s="14">
         <v>20</v>
       </c>
-      <c r="F7" s="14"/>
+      <c r="F7" s="14">
+        <v>10</v>
+      </c>
       <c r="G7" s="11">
         <f>SUM(C7:F7)</f>
-        <v>40</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="102" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="60"/>
+      <c r="A8" s="66"/>
       <c r="B8" s="7" t="s">
         <v>57</v>
       </c>
@@ -1883,11 +1911,13 @@
       <c r="E8" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="F8" s="15"/>
+      <c r="F8" s="4" t="s">
+        <v>78</v>
+      </c>
       <c r="G8" s="12"/>
     </row>
     <row r="9" spans="1:7" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="61" t="s">
+      <c r="A9" s="67" t="s">
         <v>6</v>
       </c>
       <c r="B9" s="6" t="s">
@@ -1902,14 +1932,16 @@
       <c r="E9" s="14">
         <v>5</v>
       </c>
-      <c r="F9" s="14"/>
+      <c r="F9" s="14">
+        <v>10</v>
+      </c>
       <c r="G9" s="11">
         <f>SUM(C9:F9)</f>
-        <v>11</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="62"/>
+      <c r="A10" s="68"/>
       <c r="B10" s="7" t="s">
         <v>57</v>
       </c>
@@ -1922,11 +1954,13 @@
       <c r="E10" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="F10" s="15"/>
+      <c r="F10" s="15" t="s">
+        <v>79</v>
+      </c>
       <c r="G10" s="12"/>
     </row>
     <row r="11" spans="1:7" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="63" t="s">
+      <c r="A11" s="69" t="s">
         <v>7</v>
       </c>
       <c r="B11" s="8" t="s">
@@ -1941,14 +1975,16 @@
       <c r="E11" s="16">
         <v>12</v>
       </c>
-      <c r="F11" s="16"/>
+      <c r="F11" s="16">
+        <v>12</v>
+      </c>
       <c r="G11" s="11">
         <f>SUM(C11:F11)</f>
-        <v>21</v>
+        <v>33</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="52.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="64"/>
+      <c r="A12" s="70"/>
       <c r="B12" s="7" t="s">
         <v>57</v>
       </c>
@@ -1961,11 +1997,13 @@
       <c r="E12" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="F12" s="15"/>
+      <c r="F12" s="4" t="s">
+        <v>80</v>
+      </c>
       <c r="G12" s="13"/>
     </row>
     <row r="13" spans="1:7" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A13" s="53" t="s">
+      <c r="A13" s="59" t="s">
         <v>4</v>
       </c>
       <c r="B13" s="8" t="s">
@@ -1980,14 +2018,16 @@
       <c r="E13" s="16">
         <v>5</v>
       </c>
-      <c r="F13" s="16"/>
+      <c r="F13" s="16">
+        <v>8</v>
+      </c>
       <c r="G13" s="11">
         <f>SUM(C13:F13)</f>
-        <v>9</v>
+        <v>17</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A14" s="54"/>
+      <c r="A14" s="60"/>
       <c r="B14" s="7" t="s">
         <v>57</v>
       </c>
@@ -2000,7 +2040,9 @@
       <c r="E14" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="F14" s="15"/>
+      <c r="F14" s="15" t="s">
+        <v>79</v>
+      </c>
       <c r="G14" s="13"/>
     </row>
   </sheetData>

</xml_diff>